<commit_message>
Dual Head Printing 100 mm
</commit_message>
<xml_diff>
--- a/Documentation/Experiments/Dual Head Test Prints.xlsx
+++ b/Documentation/Experiments/Dual Head Test Prints.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="12">
   <si>
     <t xml:space="preserve">Layer height</t>
   </si>
@@ -44,16 +44,19 @@
     <t xml:space="preserve">2/2</t>
   </si>
   <si>
-    <t xml:space="preserve">½</t>
+    <t xml:space="preserve">3/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4/2</t>
   </si>
   <si>
     <t xml:space="preserve">Layer deposition interval / s</t>
   </si>
   <si>
-    <t xml:space="preserve">2 on 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 on 2</t>
+    <t xml:space="preserve">Material 2 on 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Material 1 on 2</t>
   </si>
 </sst>
 </file>
@@ -414,7 +417,9 @@
   <dimension ref="A1:V14"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="14" min="1" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="14.47"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="16" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -547,10 +552,14 @@
         <v>6</v>
       </c>
       <c r="H5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
       <c r="K5" s="8" t="s">
         <v>6</v>
       </c>
@@ -561,7 +570,7 @@
         <v>6</v>
       </c>
       <c r="N5" s="8" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P5" s="4" t="n">
         <f aca="false">B5+2.4</f>
@@ -605,7 +614,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B9" s="11" t="n">
         <v>50</v>
@@ -659,7 +668,7 @@
         <v>0.55</v>
       </c>
       <c r="O9" s="13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -714,7 +723,7 @@
         <v>0.873333333333333</v>
       </c>
       <c r="O10" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -771,7 +780,7 @@
         <v>0.55</v>
       </c>
       <c r="O11" s="13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -826,7 +835,7 @@
         <v>1.70666666666667</v>
       </c>
       <c r="O12" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -883,7 +892,7 @@
         <v>0.55</v>
       </c>
       <c r="O13" s="13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -938,7 +947,7 @@
         <v>2.54</v>
       </c>
       <c r="O14" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
First batch test complete
</commit_message>
<xml_diff>
--- a/Documentation/Experiments/Dual Head Test Prints.xlsx
+++ b/Documentation/Experiments/Dual Head Test Prints.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="12">
   <si>
     <t xml:space="preserve">Layer height</t>
   </si>
@@ -203,7 +203,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -486,18 +486,42 @@
       <c r="B3" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
+      <c r="C3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>6</v>
+      </c>
       <c r="P3" s="4" t="n">
         <f aca="false">B3+2.4</f>
         <v>52.4</v>
@@ -514,18 +538,42 @@
       <c r="B4" s="7" t="n">
         <v>100</v>
       </c>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
-      <c r="L4" s="8"/>
-      <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
+      <c r="C4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="N4" s="8" t="s">
+        <v>6</v>
+      </c>
       <c r="P4" s="4" t="n">
         <f aca="false">B4+2.4</f>
         <v>102.4</v>

</xml_diff>